<commit_message>
feat(m8.1,m10,m11): nap so lieu T10/2026 den 18/10 (Zalo OA, Booking tiec, Dat ban)
- Doi ten file/thu muc T10 de nhan dung thang (OA ZALO T10.2026, Thang 10.2026)
- Booking luy ke dung lai toan bo thang; reservation.json them T10

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data_input/monthly/2025-12.xlsx
+++ b/data_input/monthly/2025-12.xlsx
@@ -633,7 +633,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   booking                   41 dòng   bắt buộc: month, status</t>
+          <t xml:space="preserve">   booking                   40 dòng   bắt buộc: month, status</t>
         </is>
       </c>
     </row>
@@ -669,7 +669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R42"/>
+  <dimension ref="A1:R41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2325,7 +2325,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Dinner</t>
+          <t>Workshop</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2335,22 +2335,27 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Lost</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>lost</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Không gian / sức chứa</t>
         </is>
       </c>
       <c r="L23" t="n">
         <v>1</v>
       </c>
       <c r="M23" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="N23" t="n">
-        <v>15000000</v>
+        <v>13860000</v>
       </c>
       <c r="O23" t="n">
         <v>1</v>
@@ -2371,24 +2376,19 @@
           <t>2025-12</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>NDC_NTMK</t>
+          <t>NCB_ET</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>NDC</t>
+          <t>NCB</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>NOIRE DINING</t>
+          <t>NOIRE ET</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2398,7 +2398,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Workshop</t>
+          <t>Room rental</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2418,17 +2418,17 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Không gian / sức chứa</t>
+          <t>Ngân sách / chi phí</t>
         </is>
       </c>
       <c r="L24" t="n">
         <v>1</v>
       </c>
       <c r="M24" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="N24" t="n">
-        <v>13860000</v>
+        <v>12000000</v>
       </c>
       <c r="O24" t="n">
         <v>1</v>
@@ -2449,19 +2449,24 @@
           <t>2025-12</t>
         </is>
       </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>NCB_ET</t>
+          <t>NDC_NTMK</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>NCB</t>
+          <t>NDC</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>NOIRE ET</t>
+          <t>NOIRE DINING</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2471,46 +2476,41 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Room rental</t>
+          <t>Dinner</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>MKT</t>
+          <t>Hotline</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Lost</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>lost</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>Ngân sách / chi phí</t>
+          <t>won</t>
         </is>
       </c>
       <c r="L25" t="n">
         <v>1</v>
       </c>
       <c r="M25" t="n">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="N25" t="n">
-        <v>12000000</v>
+        <v>10812690</v>
       </c>
       <c r="O25" t="n">
         <v>1</v>
       </c>
       <c r="P25" t="n">
-        <v>0</v>
+        <v>10812690</v>
       </c>
       <c r="Q25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R25" t="n">
         <v>0</v>
@@ -2529,17 +2529,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>NDC_NTMK</t>
+          <t>NCB_ET</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>NDC</t>
+          <t>NCB</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>NOIRE DINING</t>
+          <t>NOIRE ET</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2549,41 +2549,46 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Dinner</t>
+          <t>Meeting</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Hotline</t>
+          <t>MKT</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Lost</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>won</t>
+          <t>lost</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Ngân sách / chi phí</t>
         </is>
       </c>
       <c r="L26" t="n">
         <v>1</v>
       </c>
       <c r="M26" t="n">
-        <v>23</v>
+        <v>50</v>
       </c>
       <c r="N26" t="n">
-        <v>10812690</v>
+        <v>10000000</v>
       </c>
       <c r="O26" t="n">
         <v>1</v>
       </c>
       <c r="P26" t="n">
-        <v>10812690</v>
+        <v>0</v>
       </c>
       <c r="Q26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R26" t="n">
         <v>0</v>
@@ -2595,24 +2600,19 @@
           <t>2025-12</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>NCB_ET</t>
+          <t>NDC_NTMK</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>NCB</t>
+          <t>NDC</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>NOIRE ET</t>
+          <t>NOIRE DINING</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2627,29 +2627,24 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>MKT</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Lost</t>
+          <t>Tentative</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>lost</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>Ngân sách / chi phí</t>
+          <t>open</t>
         </is>
       </c>
       <c r="L27" t="n">
         <v>1</v>
       </c>
       <c r="M27" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="N27" t="n">
         <v>10000000</v>
@@ -2673,19 +2668,24 @@
           <t>2025-12</t>
         </is>
       </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>NDC_NTMK</t>
+          <t>NCB_ET</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>NDC</t>
+          <t>NCB</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>NOIRE DINING</t>
+          <t>NOIRE ET</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2695,17 +2695,17 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Meeting</t>
+          <t>Room rental</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>MKT</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Tentative</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -2717,7 +2717,7 @@
         <v>1</v>
       </c>
       <c r="M28" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="N28" t="n">
         <v>10000000</v>
@@ -2743,22 +2743,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>NCB_ET</t>
+          <t>NDC_NTMK</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>NCB</t>
+          <t>NDC</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>NOIRE ET</t>
+          <t>NOIRE DINING</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2768,7 +2768,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Room rental</t>
+          <t>Dinner</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -2778,19 +2778,24 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Lost</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>lost</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Ngân sách / chi phí</t>
         </is>
       </c>
       <c r="L29" t="n">
         <v>1</v>
       </c>
       <c r="M29" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="N29" t="n">
         <v>10000000</v>
@@ -2816,22 +2821,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>NDC_NTMK</t>
+          <t>NCB_ET</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>NDC</t>
+          <t>NCB</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>NOIRE DINING</t>
+          <t>NOIRE ET</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2841,34 +2846,29 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Dinner</t>
+          <t>Workshop</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>MKT</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Lost</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>lost</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>Ngân sách / chi phí</t>
+          <t>won</t>
         </is>
       </c>
       <c r="L30" t="n">
         <v>1</v>
       </c>
       <c r="M30" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="N30" t="n">
         <v>10000000</v>
@@ -2877,10 +2877,10 @@
         <v>1</v>
       </c>
       <c r="P30" t="n">
-        <v>0</v>
+        <v>10000000</v>
       </c>
       <c r="Q30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2894,37 +2894,37 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2025-12</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>NCB_ET</t>
+          <t>NDC_NTMK</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>NCB</t>
+          <t>NDC</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>NOIRE ET</t>
+          <t>NOIRE DINING</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>event</t>
+          <t>table</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Workshop</t>
+          <t>Dinner</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>MKT</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2941,16 +2941,16 @@
         <v>1</v>
       </c>
       <c r="M31" t="n">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="N31" t="n">
-        <v>10000000</v>
+        <v>8000000</v>
       </c>
       <c r="O31" t="n">
         <v>1</v>
       </c>
       <c r="P31" t="n">
-        <v>10000000</v>
+        <v>8000000</v>
       </c>
       <c r="Q31" t="n">
         <v>1</v>
@@ -2965,34 +2965,29 @@
           <t>2025-12</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>NDC_NTMK</t>
+          <t>NCB_ET</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>NDC</t>
+          <t>NCB</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>NOIRE DINING</t>
+          <t>NOIRE ET</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>table</t>
+          <t>event</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Dinner</t>
+          <t>Room rental</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -3002,31 +2997,31 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Tentative</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>won</t>
+          <t>open</t>
         </is>
       </c>
       <c r="L32" t="n">
         <v>1</v>
       </c>
       <c r="M32" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="N32" t="n">
-        <v>8000000</v>
+        <v>6000000</v>
       </c>
       <c r="O32" t="n">
         <v>1</v>
       </c>
       <c r="P32" t="n">
-        <v>8000000</v>
+        <v>0</v>
       </c>
       <c r="Q32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -3038,6 +3033,11 @@
           <t>2025-12</t>
         </is>
       </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
       <c r="C33" t="inlineStr">
         <is>
           <t>NCB_ET</t>
@@ -3060,29 +3060,29 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Room rental</t>
+          <t>Chụp hình / quay</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>MKT</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Tentative</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>won</t>
         </is>
       </c>
       <c r="L33" t="n">
         <v>1</v>
       </c>
       <c r="M33" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="N33" t="n">
         <v>6000000</v>
@@ -3091,10 +3091,10 @@
         <v>1</v>
       </c>
       <c r="P33" t="n">
-        <v>0</v>
+        <v>6000000</v>
       </c>
       <c r="Q33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -3106,11 +3106,6 @@
           <t>2025-12</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
       <c r="C34" t="inlineStr">
         <is>
           <t>NCB_ET</t>
@@ -3133,29 +3128,29 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Chụp hình / quay</t>
+          <t>Meeting</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>MKT</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>won</t>
+          <t>open</t>
         </is>
       </c>
       <c r="L34" t="n">
         <v>1</v>
       </c>
       <c r="M34" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="N34" t="n">
         <v>6000000</v>
@@ -3164,10 +3159,10 @@
         <v>1</v>
       </c>
       <c r="P34" t="n">
-        <v>6000000</v>
+        <v>0</v>
       </c>
       <c r="Q34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -3179,19 +3174,24 @@
           <t>2025-12</t>
         </is>
       </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>NCB_ET</t>
+          <t>NDC_NTMK</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>NCB</t>
+          <t>NDC</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>NOIRE ET</t>
+          <t>NOIRE DINING</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -3201,7 +3201,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Meeting</t>
+          <t>Chụp hình / quay</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -3226,7 +3226,7 @@
         <v>10</v>
       </c>
       <c r="N35" t="n">
-        <v>6000000</v>
+        <v>4000000</v>
       </c>
       <c r="O35" t="n">
         <v>1</v>
@@ -3274,22 +3274,22 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Chụp hình / quay</t>
+          <t>Meeting</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>MKT</t>
+          <t>Hotline</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Confirmed</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>won</t>
         </is>
       </c>
       <c r="L36" t="n">
@@ -3299,16 +3299,16 @@
         <v>10</v>
       </c>
       <c r="N36" t="n">
-        <v>4000000</v>
+        <v>3000000</v>
       </c>
       <c r="O36" t="n">
         <v>1</v>
       </c>
       <c r="P36" t="n">
-        <v>0</v>
+        <v>3000000</v>
       </c>
       <c r="Q36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3322,22 +3322,22 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>NDC_NTMK</t>
+          <t>NCB_ET</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>NDC</t>
+          <t>NCB</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>NOIRE DINING</t>
+          <t>NOIRE ET</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -3352,36 +3352,36 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Hotline</t>
+          <t>MKT</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>won</t>
+          <t>open</t>
         </is>
       </c>
       <c r="L37" t="n">
         <v>1</v>
       </c>
       <c r="M37" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="N37" t="n">
-        <v>3000000</v>
+        <v>0</v>
       </c>
       <c r="O37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P37" t="n">
-        <v>3000000</v>
+        <v>0</v>
       </c>
       <c r="Q37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3420,7 +3420,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Meeting</t>
+          <t>Workshop</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -3442,7 +3442,7 @@
         <v>1</v>
       </c>
       <c r="M38" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="N38" t="n">
         <v>0</v>
@@ -3503,7 +3503,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Tentative</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -3539,11 +3539,6 @@
           <t>2025-12</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
       <c r="C40" t="inlineStr">
         <is>
           <t>NCB_ET</t>
@@ -3576,7 +3571,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Tentative</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -3612,19 +3607,24 @@
           <t>2025-12</t>
         </is>
       </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>NCB_ET</t>
+          <t>NDC_NTMK</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>NCB</t>
+          <t>NDC</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>NOIRE ET</t>
+          <t>NOIRE DINING</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -3634,7 +3634,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Workshop</t>
+          <t>Dinner</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -3644,19 +3644,24 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Lost</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>lost</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Khách đổi kế hoạch / hết nhu cầu</t>
         </is>
       </c>
       <c r="L41" t="n">
         <v>1</v>
       </c>
       <c r="M41" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="N41" t="n">
         <v>0</v>
@@ -3671,84 +3676,6 @@
         <v>0</v>
       </c>
       <c r="R41" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>NDC_NTMK</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>NDC</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>NOIRE DINING</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>event</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>Dinner</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>MKT</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>Lost</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>lost</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>Khách đổi kế hoạch / hết nhu cầu</t>
-        </is>
-      </c>
-      <c r="L42" t="n">
-        <v>1</v>
-      </c>
-      <c r="M42" t="n">
-        <v>60</v>
-      </c>
-      <c r="N42" t="n">
-        <v>0</v>
-      </c>
-      <c r="O42" t="n">
-        <v>0</v>
-      </c>
-      <c r="P42" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q42" t="n">
-        <v>0</v>
-      </c>
-      <c r="R42" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>